<commit_message>
Core loop and economy: detailed design (16 features)
Gameplay, power-ups, obstacles, cell lock, level flow (pre-level, win
screen, post-win popup chain, server-side level), boosters, shop, early
offer, no-ads, choose-one pack, piggy bank, welcome back, building meta,
leaderboard and team, from the 28/10 playtest plus 07/10 shots.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/GoodsSort_ThietKeChiTiet.xlsx
+++ b/data/GoodsSort_ThietKeChiTiet.xlsx
@@ -8,19 +8,34 @@
   </bookViews>
   <sheets>
     <sheet name="Tổng quan" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="CardCollection" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="DailyQuest" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="DiggingEvents" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="EndlessTreasure" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="FoodDuel" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="GoldenGift" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="HalloweenFestival" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="LuckySpin" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="LuxuryChest" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="MasterPass" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="ScoopSquad" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="StarRush" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="WinStreak" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Boosters" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="BuildingMeta" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="CardCollection" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="CellLock" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="ChooseOnePack" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="DailyQuest" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="DiggingEvents" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="EarlyOffer" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="EndlessTreasure" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="FoodDuel" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="GameplayMechanics" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="GoldenGift" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="HalloweenFestival" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Leaderboard" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="LevelProgression" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="LuckySpin" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="LuxuryChest" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="MasterPass" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="NoAds" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="Obstacles" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="PiggyBank" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="PowerUps" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="ScoopSquad" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="Shop" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="StarRush" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="Team" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="WelcomeBack" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="WinStreak" sheetId="29" state="visible" r:id="rId29"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -450,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -502,12 +517,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Bộ sưu tập Thẻ (Collection)</t>
+          <t>Booster (Hammer/Time/x2Star)</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Bộ sưu tập thẻ — 15 bộ × 9 thẻ, mùa 60 ngày</t>
+          <t>Booster trước màn — Búa lớn, +60 giây, ×2 sao</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -525,6 +540,71 @@
         <v>2</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>[Code]  Búa lớn tự ghép 4 bộ khi vào màn, Bonus Timer +60 giây, Star Doubler ×2 sao. Mở màn 4/6/8. Mua 800 vàng.
+[Playtest]  Màn 501 cả 3 booster “vô hạn” trong 56 phút (quà Welcome Back); đồng hồ màn 05:10 → 06:10. Nút “Chơi cùng” cho cả 3 bằng một quảng cáo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Xây dựng trang trí (Building)</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Khu vực — sửa cửa hàng bằng kim cương, có cốt truyện và chọn kiểu</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>28/10/2026</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>[Playtest]  Nút “Khu vực 1” mở cảnh cửa hàng xuống cấp; bong bóng nhiệm vụ “Sửa chữa tường — Bắt đầu 100 kim cương”, thanh ngày (Day 1, 1/12) với quà cuối ngày.
+[Playtest]  Sau khi sửa có thoại cốt truyện (Sparky, Scarlet — cửa hàng của người bà) và cho chọn kiểu trang trí (3 phối màu).
+[Code]  Kim cương nhận theo độ khó màn (BuildingGemRewardByLevelSheet, 28/10 là 100/màn); chi phí task theo cỡ tiny/small/medium/large/giant; quà theo ngày.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Bộ sưu tập Thẻ (Collection)</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Bộ sưu tập thẻ — 15 bộ × 9 thẻ, mùa 60 ngày</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>28/10/2026</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>[Playtest]  Mùa cũ kết thúc 28/10 (“Bộ sưu tập mới sẽ sớm bắt đầu”), tab Bộ sưu tập đã sang album Giáng sinh: 135 thẻ, còn 59d 14h, giải lớn 10.000 vàng + bông tuyết + booster ×10.
 [Code]  15 bộ × 9 thẻ, thẻ 1–5 sao; trùng thẻ tái chế ra sao để đổi quà; gửi/nhận thẻ với bạn (giới hạn/ngày). Mở màn 41. Gói thẻ đến từ Star Rush, Food Duel, Master Pass, rương…
@@ -532,32 +612,96 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Ô khóa (Cell Lock)</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Ô khoá — kệ bị xích, số trên khoá giảm theo mỗi lần ghép</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>28/10/2026</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>[Code]  Kệ bị xích có số (mặc định 4). Mỗi match-3 ở chỗ khác giảm 1, về 0 thì xích vỡ. Mở ngay bằng goldToUnlockCellLock = 1.000 vàng hoặc xem quảng cáo.
+[Playtest]  Màn 503: 8/18 kệ bị xích “4” kèm nhãn AD (mở bằng quảng cáo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Choose One / Choose Your Gift</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Chọn một gói — 3 gói theo sự kiện + “Mua tất cả 200% giá trị”</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>28/10/2026</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>[Playtest]  Icon “%” trên Home: “Chọn một gói — Bí mật của Pharaoh”: 24.900đ (800 vàng + 5 cuốc), 49.000đ (+ rương, 10 cuốc), 69.000đ (+ 3 thẻ + rương, 30 cuốc), và Mua tất cả 99.000đ (200% giá trị).
+[Code]  Registry ChooseOnePackDataController / ChooseYourGiftDataController gắn gói vào từng sự kiện theo mùa; nội dung có bản riêng khi Collection chạy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Nhiệm vụ ngày (Daily Quest)</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Nhiệm vụ ngày — 4 nhiệm vụ, quà kèm vật phẩm sự kiện đang chạy</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
       </c>
-      <c r="D3" s="2" t="n">
+      <c r="D7" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E3" s="2" t="n">
+      <c r="E7" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="F3" s="2" t="n">
+      <c r="F7" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>[Playtest]  4 nhiệm vụ mỗi ngày (lúc chụp còn 07:00:52 tới lượt reset): đăng nhập (20 vàng), dùng vật phẩm 1 lần (Đổi chỗ ×1), tham gia 1 sự kiện (Sao ×2), hoàn thành 5 màn (50 vàng). Đủ 4/4 thì mở rương.
 [Playtest] [Code]  Phần thưởng nhiệm vụ kèm vật phẩm của sự kiện đang chạy: nhận nhiệm vụ “dùng vật phẩm” được thêm Cuốc Pharaoh ×1 (GetNumShovelWhenClaimQuest).
@@ -565,32 +709,32 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Đào báu (Dig &amp; Pharaoh)</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>Đào báu — một khuôn, nhiều giao diện (Halloween 15 màn, Pharaoh 10 màn)</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
       </c>
-      <c r="D4" s="2" t="n">
+      <c r="D8" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="E8" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="F4" s="2" t="n">
+      <c r="F8" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>[Playtest]  Hai kỳ đào chạy cùng lúc ngày 28/10: Truy tìm báu vật (Halloween, 15 màn đào) và Bí mật của Pharaoh (10 màn đào, còn 1d 22h). Cả hai dùng chung lõi DiggingBase; chỉ khác giao diện, đồ ẩn và vật phẩm (xẻng / cuốc).
 [Code] [Playtest]  Thắng màn chính được xẻng/cuốc → mỗi ô đất trong lưới 3×3 tốn 1 xẻng → tìm đủ các món ẩn theo hình bóng (một món có thể chiếm 2 ô) để qua màn đào → thanh quà ở trên có hộp quà, vàng, Freeze, rương lớn cuối.
@@ -600,32 +744,64 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Early Offer (Ưu đãi sớm)</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Ưu đãi sớm — chuỗi 5 chức danh cửa hàng, giá gạch, đếm ngược</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>28/10/2026</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>[Code]  5 bậc theo chức danh: Trainee → Junior Cashier → Shop Assistant → Store Supervisor → Shop Manager (gs_early_*), mở màn 5/6, lọc theo chiến dịch và LTV.
+[Playtest]  28/10: Store Supervisor Offer 1.500 vàng + Búa/Đũa/Đồng hồ/Đổi chỗ ×1, 299.000đ → 49.000đ (−75%), hạn 59 phút; hiện ở popup thứ 2 đầu phiên và lại hiện ở lần mở app sau (43:41, 42:35).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Kho báu Vô hạn (Endless)</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>Kho báu vô hạn — chuỗi ô quà xen kẽ miễn phí / trả phí</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
       </c>
-      <c r="D5" s="2" t="n">
+      <c r="D10" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E5" s="2" t="n">
+      <c r="E10" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="F5" s="2" t="n">
+      <c r="F10" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>[Playtest]  Chuỗi ô theo đường rắn: 100 vàng (miễn phí) → Freeze ×1 (miễn phí) → 30 phút mạng (miễn phí) → 800 vàng + Búa 99.000đ → Búa + Đồng hồ (miễn phí) → Đổi chỗ (miễn phí)… Nhận ô trước mới mở ô sau, nên ô trả phí chặn đường tới các ô miễn phí phía sau.
 [Playtest]  Kỳ cũ kết thúc thì trao bù quà chưa nhận (“Thay Kho báu vô hạn”: 100 vàng, Freeze, 30 phút mạng). Kỳ mới tự mở sau trận thắng và cả khi bấm icon SALE.
@@ -633,32 +809,32 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Trận chiến Đồ ăn (Food Duel)</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>Trận chiến đồ ăn — PvP 1-1, giao diện của Event PVP</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
       </c>
-      <c r="D6" s="2" t="n">
+      <c r="D11" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E6" s="2" t="n">
+      <c r="E11" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="F6" s="2" t="n">
+      <c r="F11" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>[Code]  Food Duel là một “skin” của Event PVP (mở màn 50, icon từ màn 40): thắng màn được bánh (vé), dùng vé ghép trận 1-1 thời gian thực qua socket, thắng nhận huy chương, leo bảng xếp hạng.
 [Playtest]  Kỳ 28/10 đã kết thúc: tổng kết “Thứ hạng của bạn 999+”, không có thưởng. Thanh huy chương: gói 2 thẻ, 100 vàng, Freeze ×1, rương lớn.
@@ -666,64 +842,98 @@
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Cơ chế sort hàng hoá</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Sort hàng 3D — ghép 3 món trên một kệ, nhiều lớp, có đồng hồ</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>28/10/2026</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>[Code] [Playtest]  Bàn là lưới kệ (Cell); mỗi kệ có nhiều lớp hàng xếp sau nhau. Chạm một món để chuyển nó sang kệ khác; đủ 3 món giống nhau trên hàng trước của một kệ thì ghép và biến mất, lộ lớp sau. Dọn sạch là thắng.
+[Code]  Thua khi hết giờ (EndGameState.TimeOut, có thể +30 giây timeAdditionEndgame) hoặc kẹt hết chỗ (Stuck). Sao thưởng = floor(thời gian còn lại / 10), ×2 khi có Star Doubler.
+[Playtest]  Màn 501: đồng hồ 05:10 (lên 06:10 sau booster thời gian), nhãn “Chuỗi x4”; màn 503 có 18 kệ với nhiều kệ bị xích (Cell Lock). Banner quảng cáo ở đáy màn hình suốt khi chơi.
+[Playtest]  Thoát giữa màn rồi mở lại thì có popup “Tiếp tục màn chơi” (lưu ván dở, LevelSavedDataController).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Golden Gift (Quà Vàng)</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>Quà vàng — thang quà theo điểm, reset 7 ngày</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
       </c>
-      <c r="D7" s="2" t="n">
+      <c r="D13" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E7" s="2" t="n">
+      <c r="E13" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="F7" s="2" t="n">
+      <c r="F13" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>[Playtest]  Thanh ngang trên cùng Home (chú chó, 0/3, 6d 7h) mở bảng Quà vàng: mốc 1 = 100 vàng, 2 = 15 phút mạng, 3 = Sao ×2 30 phút, 4 = Búa ×1…
 [Code]  Mở màn 21; điểm (point) tích bằng cách nhặt quà vàng trong màn; reset sau goldenGiftDayReset = 7 ngày. Mốc và thưởng từ GoldGiftSheet (có cột A/B và cột khi Collection chạy).</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>Lễ hội Halloween (Building)</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>Lễ hội Halloween — xây khu sự kiện bằng thuốc phép, hệ số chuỗi ×1→×20</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
       </c>
-      <c r="D8" s="2" t="n">
+      <c r="D14" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="E8" s="2" t="n">
+      <c r="E14" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="F8" s="2" t="n">
+      <c r="F14" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>[Playtest] [Code]  Sự kiện xây dựng theo mùa (lõi BaseBuildingEventDataController, dùng chung với Christmas Town Fair). Thắng màn được Bình thuốc ma thuật, nhân theo chuỗi thắng: ×1 → ×2 → ×5 → ×10 → ×20; thua một ván là về ×1.
 [Playtest]  Thuốc dùng để xây 18 hạng mục (Cổng 400, Prop 800, Máy ảnh 1.200, Khung 1.600, Căn cứ 2.000, Ghế 2.300…). Mỗi hạng mục cho bí ngô, bí ngô mở thanh quà (hộp quà, Freeze, rương) và rương lớn + khung ảnh cuối.
@@ -733,32 +943,99 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Bảng xếp hạng (Leaderboard)</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Bảng xếp hạng — Cuộc thi / Bạn / Người chơi / Đội, theo level server</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>28/10/2026</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>[Playtest]  Tab Người chơi: Thế giới / Vietnam / Cao thủ; top 1 thế giới 2.816. Tài khoản thử hiện điểm 2 (level server), dù save local ở màn 503.
+[Code]  Cuộc thi hàng tuần mở màn 12 (level_unlock_contest), thưởng theo hạng từ server.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Tiến trình màn &amp; server level</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Tiến trình màn — popup trước màn, màn thắng, chuỗi popup khi về Home</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>28/10/2026</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>[Playtest]  Popup trước màn: 3 ô Chuỗi thắng (+10/+20/+30 giây), 3 booster (Búa lớn, +thời gian, ×2 sao), nút Chơi và nút “Chơi cùng” (xem quảng cáo để có cả 3 booster), banner sự kiện đua ở đáy.
+[Playtest]  Màn thắng: kim cương (+100 mỗi màn, tiền xây Khu vực), rương mốc 5 màn (2/5, 3/5), thanh hệ số chạy ×2/×3/×5/×3/×2 với nút “Nhận ×N” bằng quảng cáo, hoặc Hoàn thành (10 vàng).
+[Playtest]  Về Home sau trận có thể mở liền: Kho báu vô hạn → Rương quý hiếm → Vòng quay may mắn → Kho báu vô hạn lần nữa; có quảng cáo xen kẽ ở lúc vào màn và sau khi thắng (từ màn 6, cách 120 giây).
+[Code] [Playtest]  Level do server quyết định: save local là 503 nhưng bảng xếp hạng vẫn ghi điểm 2 (level thật của tài khoản). Khoảng 4.500 màn baked trong APK; màn vượt mức stream từ server.
+[Playtest]  Mở game sáng 28/10 (lần đầu sau 20 ngày): Chào mừng trở lại → Store Supervisor Offer → Truy tìm báu vật → No Ads → Kho báu vô hạn (trao bù) → Lễ hội Halloween → (xem trước + luật) → Bộ sưu tập kết thúc → Home. Tức 7 popup tự mở liên tiếp, không có giới hạn kiểu 3 popup/phiên như Block Out.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>Vòng quay may mắn (Lucky Spin)</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>Vòng quay may mắn — 8 ô, quay bằng quảng cáo, ô thưởng đổi theo sự kiện</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
       </c>
-      <c r="D9" s="2" t="n">
+      <c r="D17" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E9" s="2" t="n">
+      <c r="E17" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="F9" s="2" t="n">
+      <c r="F17" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t>[Playtest]  8 ô: 100 / 250 / 500 / 1.200 vàng, Búa ×2, Đổi chỗ ×2, Đũa ×2, Freeze ×2; 2/2 lượt, mỗi lượt quay phải xem quảng cáo, reset sau ~7 giờ.
 [Code]  Mở màn 11. Ô thưởng đổi theo sự kiện đang chạy (xẻng, cuốc Pharaoh, sữa, phong bao… — cột riêng trong LuckyWheelSheet). Trọng số do server.
@@ -766,32 +1043,32 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>Luxury Chest (Rương Quý hiếm)</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>Rương quý hiếm — gom sao từ màn chơi để mở rương nối tiếp</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
       </c>
-      <c r="D10" s="2" t="n">
+      <c r="D18" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E10" s="2" t="n">
+      <c r="E18" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="F10" s="2" t="n">
+      <c r="F18" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>[Playtest]  Icon rương trên Home đếm sao: 705/1.000. Sau màn 502 vượt 1.000 thì về Home mở “Mở khóa phần thưởng”: 50 vàng + đũa sao ×1, có nút Nhận ×2 bằng quảng cáo. Rương kế cần 1.500 sao (86/1.500 → 466/1.500 sau màn 503).
 [Code]  Sao (LuxuryChestData.star) cộng từ sao thắng màn; mốc và nội dung rương do server (LuxuryChestServer), có booster/power-up ngẫu nhiên.
@@ -799,32 +1076,32 @@
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>Master Pass (battle pass)</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>Master Pass — pass tháng 30 mốc, 249.000đ, 8 lượt chơi</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
       </c>
-      <c r="D11" s="2" t="n">
+      <c r="D19" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="E11" s="2" t="n">
+      <c r="E19" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="F11" s="2" t="n">
+      <c r="F19" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G19" s="2" t="inlineStr">
         <is>
           <t>[Playtest]  “Thẻ nhiệm vụ cao cấp”, chủ đề đổi theo mùa (28/10: Halloween, còn 3d 7h). Thắng màn được chìa; 30 mốc, mỗi mốc có quà miễn phí và quà trả phí.
 [Playtest]  Kích hoạt 249.000đ (gs_master_pass_premium): mở nhánh trả phí (kể cả mốc đã qua), 8 lượt chơi thay vì 5, khung avatar và tên mạ vàng tới hết kỳ.
@@ -833,32 +1110,161 @@
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Bỏ quảng cáo (Remove Ads)</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Bỏ quảng cáo — 149.000đ + 800 vàng, chen giữa các popup sự kiện</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>28/10/2026</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>[Playtest]  Popup “Bỏ quảng cáo”: bỏ quảng cáo bắt buộc và banner, giữ quảng cáo có thưởng, tặng 800 vàng, 149.000đ. Hiện cả khi vừa bấm Tham gia sự kiện đào (chen trước màn luật).
+[Code]  Mời sau mỗi 3 quảng cáo xen kẽ (NUM_INTERSTITIAL_TO_SHOW_REMOVEADS = 3); còn có gói thuê bao Ads Subscription (tuần/tháng, 10 vé/ngày).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Vật cản (Door/Layer/Lock...)</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Vật cản — rào cản, bom, lớp ẩn, kệ đóng, ô kẹt</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>28/10/2026</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>[Code]  Mechanic theo màn: ReverseItem, LockSlot, CloseCellEnd, BombItem (60 giây), HiddenLayerItem, LockedItem, cộng Cell Lock. Mỗi loại có màn tutorial riêng.
+[Playtest]  Màn 501 hiện tooltip “Rào cản ngăn chặn vật thể di chuyển!” với nút Đã hiểu ngay khi vào màn.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Heo vàng (Piggy Bank)</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Heo vàng — mỗi màn nạp vàng, đầy thì mua để đập</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>28/10/2026</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>[Playtest]  Icon heo: 100/1.500 → 200/1.500 (+100 mỗi màn thắng); popup có mốc 1.000 và 1.500, nhãn −35%.
+[Code]  goldPerLevel, goldMax, giá và % giảm theo loại heo gán theo LTV (Free/Minnow/Dolphin/Whale); đầy thì cooldown 24 giờ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Power-up trong màn (Hammer/Freeze/Wand/Swap)</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Power-up trong màn — Búa, Đóng băng, Đũa, Đổi chỗ; hết thì 500 vàng hoặc quảng cáo</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>28/10/2026</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>[Code]  Búa (tự ghép 1 bộ / phá bom), Đóng băng (dừng đồng hồ 15 giây), Đũa (biến 9 món thành 3 bộ), Đổi chỗ (xáo toàn bàn). Mở ở màn 2 / 9 / 6 / 4 (A/B FTUE đổi được).
+[Playtest]  Hết thì popup “Nhận thêm”: 1 cái = 500 vàng hoặc Miễn phí (xem quảng cáo). Mua bằng vàng là dùng ngay.
+[Playtest]  Dùng Búa liên tục dọn được cả màn (playtest dùng cách này để vượt màn 501–503, khoảng 50–150 lần mỗi màn vì có nhiều lớp).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>Biệt đội bán Kem (Scoop)</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>Biệt đội bán kem — sự kiện hợp tác 4 người: sữa → vòng quay → muỗng kem</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
       </c>
-      <c r="D12" s="2" t="n">
+      <c r="D24" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="E12" s="2" t="n">
+      <c r="E24" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="F12" s="2" t="n">
+      <c r="F24" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr">
         <is>
           <t>[Playtest] [Code]  Code gọi là Star Collaboration, mở màn 41. Mời tối đa 4 bạn/đồng đội vào biệt đội. Thắng màn được Sữa → dùng sữa quay vòng quay → ra Muỗng kem → muỗng tích vào các món kem chung của cả nhóm.
 [Playtest]  Hoàn thành mọi món kem thì nhận giải lớn: rương + khung avatar kem (frame_id −2).
@@ -867,32 +1273,65 @@
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Cửa hàng (Shop)</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Cửa hàng — offer cá nhân −95%, pass, bundle, coin</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>28/10/2026</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>[Playtest]  Thứ tự từ trên xuống (28/10): “Chỉ dành cho bạn” −95% (2.000 vàng + booster ×2, 589.000đ → 24.900đ, đếm ngược 23:57) → thẻ Master Pass 249.000đ → Tân thủ −90% → Gói Hiếm 149.000đ (−70%) → Bỏ quảng cáo 149.000đ (+800 vàng) → Gói Lớn 169.000đ → Siêu cấp 1.290.000đ → Huyền thoại 2.390.000đ (“Giá trị nhất”) → coin: 80 miễn phí (quảng cáo), 1.000 = 49.000đ, 2.600 = 129.000đ…
+[Nhận định]  Offer cá nhân đặt trên cùng với giá gạch 589.000đ và đồng hồ 24 giờ: neo giá rất mạnh. Icon của nó (23:58) xuất hiện trên Home sau trận thắng thứ 3 trong phiên; điều kiện kích hoạt chính xác chưa xác minh.
+[Code]  Danh sách bundle lọc theo RemoteConfig (CheckShopBundleTypeFromRemoteConfig); vàng miễn phí qua quảng cáo 80 mỗi 300 giây.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>Cuộc đua kiếm Sao (Star Rush)</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>Cuộc đua kiếm sao — 1 giờ, 5 người, bot mô phỏng trên máy</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C26" s="2" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
       </c>
-      <c r="D13" s="2" t="n">
+      <c r="D26" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E13" s="2" t="n">
+      <c r="E26" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="F13" s="2" t="n">
+      <c r="F26" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="G26" s="2" t="inlineStr">
         <is>
           <t>[Playtest]  Mở từ màn 15. Bấm Chơi thì bắt đầu một vòng 1 giờ với 4 đối thủ; ai có nhiều sao nhất khi hết giờ thì thắng. Quà hạng 1: gói 6 thẻ + 200 vàng + Búa + Đồng hồ.
 [Code]  Đối thủ là bot mô phỏng trên client: StarRushDataController sinh bot (loại casual/silent, tier sức mạnh) và tăng sao theo thời gian bằng các khoảng cố định trong code (50–100, 100–140, 130–170, 300–400…). Khác Block Out, nơi bot do server tính.
@@ -901,32 +1340,97 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Team / Đội (clan)</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Đội — tối đa 50 người, xin/tặng tim, nền cho sự kiện nhóm</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>28/10/2026</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>[Playtest]  Tab Đội: Tham gia / Tìm kiếm / Tạo mới; danh sách đội 6–49/50 thành viên. Mất mạng thì báo “Mất kết nối, đang cố gắng kết nối lại”.
+[Code]  Mở màn 11, tạo đội 100 vàng, tặng tim tối đa 5 mỗi yêu cầu, dữ liệu qua socket UDP; là nền cho Scoop Squad, Delivery Battle, Team Treasure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Welcome Back (Chào mừng trở lại)</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Chào mừng trở lại — quà khi vắng ≥ 7 ngày, rồi chuỗi offer</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>28/10/2026</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>[Playtest]  Mở lại sau 20 ngày: popup “Chào mừng trở lại” với 6 món: 100 vàng, 5 phút booster thời gian, 5 phút Búa, 5 phút ×2 sao, 15 phút mạng vô hạn, Freeze ×1. Nhờ đó vào màn với booster vô hạn.
+[Code]  Kích hoạt khi vắng numDayToActiveWelcomeBack = 7 ngày; sau 3 màn mở thêm gói “Raise Sparky Up” (free 24h / paid 48h).
+[Playtest]  Mở game sáng 28/10 (lần đầu sau 20 ngày): Chào mừng trở lại → Store Supervisor Offer → Truy tìm báu vật → No Ads → Kho báu vô hạn (trao bù) → Lễ hội Halloween → (xem trước + luật) → Bộ sưu tập kết thúc → Home. Tức 7 popup tự mở liên tiếp, không có giới hạn kiểu 3 popup/phiên như Block Out.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
         <is>
           <t>Chuỗi thắng (Win Streak)</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B29" s="2" t="inlineStr">
         <is>
           <t>Chuỗi thắng — +10 / +20 / +30 giây cho màn kế</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C29" s="2" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
       </c>
-      <c r="D14" s="2" t="n">
+      <c r="D29" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E14" s="2" t="n">
+      <c r="E29" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="F14" s="2" t="n">
+      <c r="F29" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G29" s="2" t="inlineStr">
         <is>
           <t>[Code]  Mở màn 12 (13 nếu A/B FTUE). Mỗi màn thắng +1 chuỗi (tối đa 3); màn kế được cộng streak × 10 giây. Thua là về 0.
 [Playtest]  Popup trước màn hiện 3 ô đồng hồ +10s / +20s / +30s với nhãn Chuỗi thắng 1/2/3 sáng dần. Home hiện “Chuỗi thắng 3” ngay trên nút Màn.
@@ -959,7 +1463,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Luxury Chest (Rương Quý hiếm) — Rương quý hiếm — gom sao từ màn chơi để mở rương nối tiếp (28/10/2026)</t>
+          <t>Kho báu Vô hạn (Endless) — Kho báu vô hạn — chuỗi ô quà xen kẽ miễn phí / trả phí (28/10/2026)</t>
         </is>
       </c>
     </row>
@@ -1001,17 +1505,17 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Xem rương</t>
+          <t>Trao bù kỳ cũ</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Giao diện</t>
+          <t>Client</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Popup Rương quý hiếm 705/1.000.</t>
+          <t>Popup quà chưa nhận.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -1021,7 +1525,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>LuxuryChest/01_popup_705_1000</t>
+          <t>EndlessTreasure/01_unclaimed_rewards</t>
         </is>
       </c>
     </row>
@@ -1031,17 +1535,17 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Đủ sao → mở</t>
+          <t>Chuỗi kỳ mới</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Client</t>
+          <t>Giao diện</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Về Home: Mở khóa phần thưởng, Nhận ×2 (quảng cáo) hoặc Nhận.</t>
+          <t>Tự mở sau trận; nhận ô đầu thì chuỗi dịch lên.</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -1051,7 +1555,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>LuxuryChest/02_chest_opened, LuxuryChest/03_next_tier_86_1500</t>
+          <t>EndlessTreasure/02_chain_on_return, EndlessTreasure/03_claim_first, EndlessTreasure/05_auto_open_again</t>
         </is>
       </c>
     </row>
@@ -1065,7 +1569,7 @@
     <row r="8">
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Biến tiền tệ “điểm” (sao) thành rương nối tiếp vô hạn với mốc tăng dần; thêm nút ×2 quảng cáo ở lúc mở để kiếm doanh thu quảng cáo.</t>
+          <t>Xen ô trả phí giữa chuỗi quà miễn phí: người chơi đã nhận vài ô miễn phí sẽ thấy “mua một ô để mở tiếp” rất hợp lý.</t>
         </is>
       </c>
     </row>
@@ -1075,6 +1579,1299 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="90" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Trận chiến Đồ ăn (Food Duel) — Trận chiến đồ ăn — PvP 1-1, giao diện của Event PVP (28/10/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>Bước</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>Ai</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>Mô tả</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>Bằng chứng</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>Ảnh</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Tổng kết kỳ</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Giao diện</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Popup Tổng kết thứ hạng: 999+, phần thưởng “--”.</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>[Playtest]</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>FoodDuel/01_season_result</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Bảng sự kiện</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Giao diện</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Huy chương 0, thanh quà, cảnh đấu xanh–đỏ.</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>[Playtest]</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>FoodDuel/02_board_ended, FoodDuel/03_info</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Vận dụng cho game khác</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Tách lõi PvP khỏi giao diện để đổi chủ đề theo mùa (Food Duel, Punch Clash…) mà không làm lại matchmaking.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Cấm vật phẩm dừng thời gian trong PvP thời gian thực để giữ công bằng.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="90" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Cơ chế sort hàng hoá — Sort hàng 3D — ghép 3 món trên một kệ, nhiều lớp, có đồng hồ (28/10/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>Bước</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>Ai</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>Mô tả</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>Bằng chứng</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>Ảnh</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Vào màn</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Người chơi</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Popup trước màn → bàn chơi; lần đầu gặp vật cản có tooltip (Rào cản).</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>[Playtest]</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>GameplayMechanics/01_board, GameplayMechanics/02_board_start</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Ghép</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Người chơi</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Mỗi bộ 3 ghép xong thì cộng sao trên HUD; dùng Búa để tự ghép 1 bộ.</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>[Playtest]</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>GameplayMechanics/03_hammer1</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Thắng</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Màn hình “Cấp độ N đã hoàn thành”: kim cương, rương mốc 5 màn, sao, heo đất.</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>[Playtest]</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>LevelProgression/06_win_popup_ad_multiplier, LevelProgression/10_win_503_star_piggy</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Vận dụng cho game khác</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Nhiều lớp hàng sau một kệ cho độ sâu mà vẫn giữ thao tác một chạm; vật cản (xích, rào, bom) chỉ cần đổi luật ở cấp kệ.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="90" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Golden Gift (Quà Vàng) — Quà vàng — thang quà theo điểm, reset 7 ngày (28/10/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>Bước</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>Ai</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>Mô tả</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>Bằng chứng</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>Ảnh</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Bảng Quà vàng</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Giao diện</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>4 mốc đầu đều khoá, thanh 0/3.</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>[Playtest]</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>GoldenGift/01_track</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Vận dụng cho game khác</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Đặt thanh tiến độ “quà miễn phí” ở vị trí nổi nhất trên Home để người chơi luôn thấy mình sắp nhận gì.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="90" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Lễ hội Halloween (Building) — Lễ hội Halloween — xây khu sự kiện bằng thuốc phép, hệ số chuỗi ×1→×20 (28/10/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>Bước</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>Ai</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>Mô tả</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>Bằng chứng</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>Ảnh</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Mời tham gia</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Giao diện</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Popup Lễ hội Halloween 4d 22h, Tham gia.</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>[Playtest]</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>HalloweenFestival/01_join_popup</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Xem trước khu hoàn chỉnh</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Giao diện</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Cảnh khu lễ hội đã trang trí đủ, ghi chú “Xem trước trang trí”.</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>[Playtest]</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>HalloweenFestival/02_preview_finished_area</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Luật</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Giao diện</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Thu thuốc từ các màn → xây khu → nhận bí ngô → nhận thưởng; dải hệ số ×1…×20, thua về ×1.</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>[Playtest]</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>HalloweenFestival/03_how_to_play</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Bảng xây</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Người chơi</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Số thuốc hiện có, hệ số hiện tại, lưới hạng mục có giá thuốc, thanh quà bí ngô phía trên.</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>[Playtest]</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>HalloweenFestival/04_build_board, HalloweenFestival/05_area_before_build</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Kỳ đã kết thúc</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Giao diện</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Một kỳ cũ cùng loại vẫn còn icon “Đã kết thúc” tới khi người chơi mở xem; xem xong icon biến mất.</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>[Playtest]</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>HalloweenFestival/06_ended_instance</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Hạng mục đầu (quan sát)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>Hạng mục</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="inlineStr">
+        <is>
+          <t>Thuốc</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Cổng</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Prop</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Máy ảnh</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Khung</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>1600</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Căn cứ</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Ghế</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>2300</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>[Code]  18 hạng mục (numItems), giá và bí ngô thưởng từ BuildingHalloweenStepBuildSheet (server).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Vận dụng cho game khác</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Cho người chơi xem trước khu hoàn chỉnh ngay khi tham gia: mục tiêu trực quan rõ hơn mọi thanh tiến độ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Gắn hệ số chuỗi thắng vào tiền tệ sự kiện (thuốc) để mỗi trận thắng liền mạch đáng giá gấp nhiều lần.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="90" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Bảng xếp hạng (Leaderboard) — Bảng xếp hạng — Cuộc thi / Bạn / Người chơi / Đội, theo level server (28/10/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>Bước</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>Ai</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>Mô tả</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>Bằng chứng</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>Ảnh</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Tab</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Người chơi</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Top thế giới.</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>[Playtest]</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Leaderboard/01_tab</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="90" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Tiến trình màn &amp; server level — Tiến trình màn — popup trước màn, màn thắng, chuỗi popup khi về Home (28/10/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>Bước</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>Ai</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>Mô tả</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>Bằng chứng</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>Ảnh</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Trước màn</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Giao diện</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Chuỗi thắng, booster, Chơi / Chơi cùng (AD).</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>[Playtest]</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>LevelProgression/01_prelevel</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Ván dở</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Giao diện</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Mở lại app giữa màn: Tiếp tục màn chơi / Từ bỏ.</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>[Playtest]</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>LevelProgression/05_resume_level_popup</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Thắng</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Kim cương, rương mốc, thanh hệ số quảng cáo.</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>[Playtest]</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>LevelProgression/06_win_popup_ad_multiplier, LevelProgression/10_win_503_star_piggy</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Về Home</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Chuỗi popup sau trận.</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>[Playtest]</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>EndlessTreasure/02_chain_on_return, LuxuryChest/02_chest_opened, LuckySpin/02_auto_open_on_return</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Bảng xếp hạng thấy level server</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Giao diện</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Điểm của tài khoản thử = 2 dù local ở màn 503.</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>[Playtest]</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Leaderboard/01_tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Vận dụng cho game khác</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Màn thắng có thanh hệ số “dừng ở đâu nhận ×N bằng quảng cáo”: biến phần thưởng nhỏ thành một lượt xem rewarded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>[Nhận định]  Chuỗi popup không giới hạn kéo dài thời gian từ lúc thắng tới lúc chơi màn kế; Block Out giới hạn 2 popup mỗi lượt về Home để tránh việc này.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="90" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Vòng quay may mắn (Lucky Spin) — Vòng quay may mắn — 8 ô, quay bằng quảng cáo, ô thưởng đổi theo sự kiện (28/10/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>Bước</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>Ai</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>Mô tả</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>Bằng chứng</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>Ảnh</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Vòng quay</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Giao diện</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Mở từ icon và tự mở sau trận.</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>[Playtest]</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>LuckySpin/01_wheel_ad_spin, LuckySpin/02_auto_open_on_return</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Vận dụng cho game khác</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Vòng quay thưởng quảng cáo là nguồn rewarded ổn định; đổi ô thưởng sang vật phẩm sự kiện để nó phục vụ sự kiện đang chạy.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="90" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Luxury Chest (Rương Quý hiếm) — Rương quý hiếm — gom sao từ màn chơi để mở rương nối tiếp (28/10/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>Bước</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>Ai</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>Mô tả</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>Bằng chứng</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>Ảnh</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Xem rương</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Giao diện</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Popup Rương quý hiếm 705/1.000.</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>[Playtest]</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>LuxuryChest/01_popup_705_1000</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Đủ sao → mở</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Về Home: Mở khóa phần thưởng, Nhận ×2 (quảng cáo) hoặc Nhận.</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>[Playtest]</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>LuxuryChest/02_chest_opened, LuxuryChest/03_next_tier_86_1500</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Vận dụng cho game khác</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Biến tiền tệ “điểm” (sao) thành rương nối tiếp vô hạn với mốc tăng dần; thêm nút ×2 quảng cáo ở lúc mở để kiếm doanh thu quảng cáo.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1342,7 +3139,476 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="90" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Booster (Hammer/Time/x2Star) — Booster trước màn — Búa lớn, +60 giây, ×2 sao (28/10/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>Bước</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>Ai</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>Mô tả</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>Bằng chứng</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>Ảnh</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Chọn booster</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Giao diện</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Popup trước màn.</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>[Playtest]</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>LevelProgression/01_prelevel, @gs_mech_lvl5_a.jpg</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="90" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Bỏ quảng cáo (Remove Ads) — Bỏ quảng cáo — 149.000đ + 800 vàng, chen giữa các popup sự kiện (28/10/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>Bước</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>Ai</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>Mô tả</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>Bằng chứng</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>Ảnh</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Popup</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Giao diện</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Bỏ quảng cáo 149.000đ.</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>[Playtest]</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>NoAds/01_popup_over_event</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="90" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Vật cản (Door/Layer/Lock...) — Vật cản — rào cản, bom, lớp ẩn, kệ đóng, ô kẹt (28/10/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>Bước</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>Ai</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>Mô tả</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>Bằng chứng</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>Ảnh</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Giới thiệu</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Giao diện</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Tooltip rào cản, ảnh 07/10 kệ giới hạn.</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>[Playtest]</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Obstacles/01_barrier_intro, @gs_lv7_b.jpg</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="90" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Heo vàng (Piggy Bank) — Heo vàng — mỗi màn nạp vàng, đầy thì mua để đập (28/10/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>Bước</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>Ai</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>Mô tả</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>Bằng chứng</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>Ảnh</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Popup heo</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Giao diện</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>200 vàng trong heo.</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>[Playtest]</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>PiggyBank/01_piggy_200, LevelProgression/10_win_503_star_piggy</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="90" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Power-up trong màn (Hammer/Freeze/Wand/Swap) — Power-up trong màn — Búa, Đóng băng, Đũa, Đổi chỗ; hết thì 500 vàng hoặc quảng cáo (28/10/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>Bước</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>Ai</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>Mô tả</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>Bằng chứng</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>Ảnh</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Hết power-up</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Giao diện</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Popup Nhận thêm Búa ×1: 500 vàng hoặc quảng cáo.</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>[Playtest]</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>PowerUps/01_buy_more_hammer, @sp_powerup_hammer.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Vận dụng cho game khác</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Cho mua power-up lẻ ngay trong màn với giá vàng thấp và lựa chọn quảng cáo song song: hai đường đều kéo người chơi ở lại màn.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1514,7 +3780,128 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="90" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Cửa hàng (Shop) — Cửa hàng — offer cá nhân −95%, pass, bundle, coin (28/10/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>Bước</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>Ai</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>Mô tả</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>Bằng chứng</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>Ảnh</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Cuộn Shop</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Người chơi</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Ba ảnh từ trên xuống.</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>[Playtest]</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Shop/01_top, Shop/02_mid, Shop/03_low</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Thanh toán</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Giao diện</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>07/10: bảng Google Play thật, huỷ thì “Đã huỷ”.</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>[Playtest]</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>@gs_201_buysheet.jpg, @gs_210_afterShopBack.jpg</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1772,7 +4159,203 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="90" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Team / Đội (clan) — Đội — tối đa 50 người, xin/tặng tim, nền cho sự kiện nhóm (28/10/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>Bước</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>Ai</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>Mô tả</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>Bằng chứng</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>Ảnh</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Danh sách đội</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Người chơi</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Tham gia đội.</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>[Playtest]</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Team/01_tab</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="90" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Welcome Back (Chào mừng trở lại) — Chào mừng trở lại — quà khi vắng ≥ 7 ngày, rồi chuỗi offer (28/10/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>Bước</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>Ai</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>Mô tả</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>Bằng chứng</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>Ảnh</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Quà quay lại</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Giao diện</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Popup đầu tiên của phiên.</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>[Playtest]</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>WelcomeBack/01_popup, EarlyOffer/01_store_supervisor_offer, DiggingEvents/01_join_popup</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Vận dụng cho game khác</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Tặng booster vô hạn theo phút khi người chơi quay lại: trận đầu dễ thắng, tạo cảm giác “vẫn giỏi”.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1899,111 +4482,6 @@
       <c r="B8" s="2" t="inlineStr">
         <is>
           <t>Thưởng chuỗi thắng bằng thời gian cho màn kế: rẻ, dễ hiểu, và hợp với game có đồng hồ.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="90" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>Bộ sưu tập Thẻ (Collection) — Bộ sưu tập thẻ — 15 bộ × 9 thẻ, mùa 60 ngày (28/10/2026)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B3" s="1" t="inlineStr">
-        <is>
-          <t>Bước</t>
-        </is>
-      </c>
-      <c r="C3" s="1" t="inlineStr">
-        <is>
-          <t>Ai</t>
-        </is>
-      </c>
-      <c r="D3" s="1" t="inlineStr">
-        <is>
-          <t>Mô tả</t>
-        </is>
-      </c>
-      <c r="E3" s="1" t="inlineStr">
-        <is>
-          <t>Bằng chứng</t>
-        </is>
-      </c>
-      <c r="F3" s="1" t="inlineStr">
-        <is>
-          <t>Ảnh</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Hết mùa → mùa mới</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Giao diện</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Popup kết thúc mùa, rồi album Giáng sinh.</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>[Playtest]</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>CardCollection/01_season_ended, CardCollection/02_new_christmas_album</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>Vận dụng cho game khác</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Album dài 60 ngày làm “sink” chung cho gói thẻ từ mọi sự kiện; mở mùa mới ngay khi mùa cũ hết để không có khoảng trống.</t>
         </is>
       </c>
     </row>
@@ -2032,7 +4510,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Nhiệm vụ ngày (Daily Quest) — Nhiệm vụ ngày — 4 nhiệm vụ, quà kèm vật phẩm sự kiện đang chạy (28/10/2026)</t>
+          <t>Xây dựng trang trí (Building) — Khu vực — sửa cửa hàng bằng kim cương, có cốt truyện và chọn kiểu (28/10/2026)</t>
         </is>
       </c>
     </row>
@@ -2074,17 +4552,17 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Danh sách</t>
+          <t>Khu vực</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Giao diện</t>
+          <t>Người chơi</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>4 nhiệm vụ, thanh rương 0/4, đồng hồ 07:00:52.</t>
+          <t>Cảnh và nhiệm vụ.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -2094,7 +4572,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>DailyQuest/01_list</t>
+          <t>BuildingMeta/01_area, BuildingMeta/02_task_repair_wall</t>
         </is>
       </c>
     </row>
@@ -2104,17 +4582,17 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Nhận</t>
+          <t>Cốt truyện và kiểu</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Người chơi</t>
+          <t>Giao diện</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Chúc mừng: Đổi chỗ ×1 + Cuốc ×1.</t>
+          <t>Thoại, nhật ký thoại, chọn phối màu.</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -2124,7 +4602,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>DailyQuest/02_claim_with_event_token</t>
+          <t>BuildingMeta/03_story_dialogue, BuildingMeta/04_dialogue_log, BuildingMeta/05_choose_style, BuildingMeta/06_story_continues</t>
         </is>
       </c>
     </row>
@@ -2138,7 +4616,7 @@
     <row r="8">
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Cho nhiệm vụ ngày rót tiền tệ của sự kiện đang chạy: người chơi chỉ làm nhiệm vụ cũng tiến được trong sự kiện.</t>
+          <t>Meta trang trí có cốt truyện + chọn kiểu (công thức Homescapes) cho mỗi màn thắng một ý nghĩa dài hạn ngoài sự kiện.</t>
         </is>
       </c>
     </row>
@@ -2153,7 +4631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2167,7 +4645,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Đào báu (Dig &amp; Pharaoh) — Đào báu — một khuôn, nhiều giao diện (Halloween 15 màn, Pharaoh 10 màn) (28/10/2026)</t>
+          <t>Bộ sưu tập Thẻ (Collection) — Bộ sưu tập thẻ — 15 bộ × 9 thẻ, mùa 60 ngày (28/10/2026)</t>
         </is>
       </c>
     </row>
@@ -2209,7 +4687,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Mời tham gia</t>
+          <t>Hết mùa → mùa mới</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -2219,7 +4697,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Popup chủ đề (Halloween / Pharaoh) với đồng hồ và nút Tham gia; tự mở trong chuỗi popup đầu phiên.</t>
+          <t>Popup kết thúc mùa, rồi album Giáng sinh.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -2229,264 +4707,21 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>DiggingEvents/01_join_popup, DiggingEvents/10_pharaoh_join</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Luật 4 bước</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Giao diện</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Thắng màn → thu cuốc/xẻng → tìm đồ ẩn → giành phần thưởng.</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>[Playtest]</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>DiggingEvents/08_info, DiggingEvents/11_pharaoh_how_to</t>
+          <t>CardCollection/01_season_ended, CardCollection/02_new_christmas_album</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Bàn đào</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Người chơi</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>Màn 1/15 (Halloween) hoặc 1/10 (Pharaoh): khung trên là hình bóng món cần tìm, lưới đất 3×3, số xẻng ở dưới, thanh quà ở trên.</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>[Playtest]</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>DiggingEvents/04_dig_board, DiggingEvents/12_pharaoh_board</t>
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Vận dụng cho game khác</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n">
-        <v>4</v>
-      </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Đào</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Người chơi</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>Mỗi chạm tốn 1 xẻng; ô thứ hai lộ một nửa viên kẹo (món chiếm 2 ô).</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>[Playtest]</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>DiggingEvents/05_dig_one, DiggingEvents/06_dig_two</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Hết xẻng → shop</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Giao diện</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Bấm “+”: 3 gói xẻng 49k / 129k / 249k.</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>[Playtest]</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>DiggingEvents/07_buy_shovel</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Hết kỳ</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Giao diện</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>“Đã kết thúc — hãy đào ngay”: vẫn vào đào bằng xẻng còn lại.</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>[Playtest]</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>DiggingEvents/03_ended_dig_now</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>Kinh tế đào (quan sát 28/10)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t>Mục</t>
-        </is>
-      </c>
-      <c r="B12" s="1" t="inlineStr">
-        <is>
-          <t>Giá trị</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Số màn đào</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>Halloween 15, Pharaoh 10</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>Chi phí</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>1 xẻng/cuốc mỗi ô</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>Gói xẻng</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>×10 49.000đ · ×30 129.000đ · ×60 249.000đ</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>Gói Pharaoh “chọn một”</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>24.900đ (800 vàng + 5 cuốc) · 49.000đ (+ rương, 10 cuốc) · 69.000đ (+ 3 thẻ, 30 cuốc) · mua tất cả 99.000đ</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Nguồn xẻng/cuốc</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>thắng màn, nhiệm vụ ngày, vòng quay may mắn, gói IAP</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>Vận dụng cho game khác</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>Viết lõi sự kiện một lần (DiggingBase) rồi đổi giao diện theo mùa: cùng lúc chạy được 2 kỳ (Halloween + Pharaoh) mà không thêm logic.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>Cho phần thưởng nhỏ khi đào trượt và cho dùng xẻng dư sau khi kỳ kết thúc: giảm cảm giác “phí tiền mua xẻng”.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>Rót vật phẩm sự kiện vào mọi nguồn khác (nhiệm vụ ngày, vòng quay) để người không mua vẫn tiến được.</t>
+          <t>Album dài 60 ngày làm “sink” chung cho gói thẻ từ mọi sự kiện; mở mùa mới ngay khi mùa cũ hết để không có khoảng trống.</t>
         </is>
       </c>
     </row>
@@ -2496,6 +4731,216 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="90" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Ô khóa (Cell Lock) — Ô khoá — kệ bị xích, số trên khoá giảm theo mỗi lần ghép (28/10/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>Bước</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>Ai</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>Mô tả</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>Bằng chứng</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>Ảnh</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Bàn có ô khoá</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Giao diện</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Màn 503 và ảnh màn 5 ngày 07/10.</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>[Playtest]</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>CellLock/01_locked_shelves_l503, @gs_mech_lvl5_b.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Vận dụng cho game khác</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Vật cản “tự mở sau N lần ghép” kèm lối tắt trả vàng/quảng cáo: không chặn người chơi, nhưng tạo một điểm bán.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="90" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Choose One / Choose Your Gift — Chọn một gói — 3 gói theo sự kiện + “Mua tất cả 200% giá trị” (28/10/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>Bước</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>Ai</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>Mô tả</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>Bằng chứng</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>Ảnh</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Popup</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Giao diện</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>3 gói + mua tất cả.</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>[Playtest]</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>ChooseOnePack/01_pharaoh_choose_one</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Vận dụng cho game khác</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Bán 3 gói giá tăng dần và một nút “mua tất cả” rẻ hơn tổng (142.900đ → 99.000đ) để đẩy người chơi lên mức chi cao nhất.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2515,7 +4960,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Kho báu Vô hạn (Endless) — Kho báu vô hạn — chuỗi ô quà xen kẽ miễn phí / trả phí (28/10/2026)</t>
+          <t>Nhiệm vụ ngày (Daily Quest) — Nhiệm vụ ngày — 4 nhiệm vụ, quà kèm vật phẩm sự kiện đang chạy (28/10/2026)</t>
         </is>
       </c>
     </row>
@@ -2557,17 +5002,17 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Trao bù kỳ cũ</t>
+          <t>Danh sách</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Client</t>
+          <t>Giao diện</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Popup quà chưa nhận.</t>
+          <t>4 nhiệm vụ, thanh rương 0/4, đồng hồ 07:00:52.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -2577,7 +5022,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>EndlessTreasure/01_unclaimed_rewards</t>
+          <t>DailyQuest/01_list</t>
         </is>
       </c>
     </row>
@@ -2587,17 +5032,17 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Chuỗi kỳ mới</t>
+          <t>Nhận</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Giao diện</t>
+          <t>Người chơi</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Tự mở sau trận; nhận ô đầu thì chuỗi dịch lên.</t>
+          <t>Chúc mừng: Đổi chỗ ×1 + Cuốc ×1.</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -2607,7 +5052,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>EndlessTreasure/02_chain_on_return, EndlessTreasure/03_claim_first, EndlessTreasure/05_auto_open_again</t>
+          <t>DailyQuest/02_claim_with_event_token</t>
         </is>
       </c>
     </row>
@@ -2621,254 +5066,7 @@
     <row r="8">
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Xen ô trả phí giữa chuỗi quà miễn phí: người chơi đã nhận vài ô miễn phí sẽ thấy “mua một ô để mở tiếp” rất hợp lý.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="90" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>Trận chiến Đồ ăn (Food Duel) — Trận chiến đồ ăn — PvP 1-1, giao diện của Event PVP (28/10/2026)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B3" s="1" t="inlineStr">
-        <is>
-          <t>Bước</t>
-        </is>
-      </c>
-      <c r="C3" s="1" t="inlineStr">
-        <is>
-          <t>Ai</t>
-        </is>
-      </c>
-      <c r="D3" s="1" t="inlineStr">
-        <is>
-          <t>Mô tả</t>
-        </is>
-      </c>
-      <c r="E3" s="1" t="inlineStr">
-        <is>
-          <t>Bằng chứng</t>
-        </is>
-      </c>
-      <c r="F3" s="1" t="inlineStr">
-        <is>
-          <t>Ảnh</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Tổng kết kỳ</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Giao diện</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Popup Tổng kết thứ hạng: 999+, phần thưởng “--”.</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>[Playtest]</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>FoodDuel/01_season_result</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Bảng sự kiện</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Giao diện</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Huy chương 0, thanh quà, cảnh đấu xanh–đỏ.</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>[Playtest]</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>FoodDuel/02_board_ended, FoodDuel/03_info</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>Vận dụng cho game khác</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Tách lõi PvP khỏi giao diện để đổi chủ đề theo mùa (Food Duel, Punch Clash…) mà không làm lại matchmaking.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Cấm vật phẩm dừng thời gian trong PvP thời gian thực để giữ công bằng.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="90" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>Golden Gift (Quà Vàng) — Quà vàng — thang quà theo điểm, reset 7 ngày (28/10/2026)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B3" s="1" t="inlineStr">
-        <is>
-          <t>Bước</t>
-        </is>
-      </c>
-      <c r="C3" s="1" t="inlineStr">
-        <is>
-          <t>Ai</t>
-        </is>
-      </c>
-      <c r="D3" s="1" t="inlineStr">
-        <is>
-          <t>Mô tả</t>
-        </is>
-      </c>
-      <c r="E3" s="1" t="inlineStr">
-        <is>
-          <t>Bằng chứng</t>
-        </is>
-      </c>
-      <c r="F3" s="1" t="inlineStr">
-        <is>
-          <t>Ảnh</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Bảng Quà vàng</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Giao diện</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>4 mốc đầu đều khoá, thanh 0/3.</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>[Playtest]</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>GoldenGift/01_track</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>Vận dụng cho game khác</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Đặt thanh tiến độ “quà miễn phí” ở vị trí nổi nhất trên Home để người chơi luôn thấy mình sắp nhận gì.</t>
+          <t>Cho nhiệm vụ ngày rót tiền tệ của sự kiện đang chạy: người chơi chỉ làm nhiệm vụ cũng tiến được trong sự kiện.</t>
         </is>
       </c>
     </row>
@@ -2897,7 +5095,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Lễ hội Halloween (Building) — Lễ hội Halloween — xây khu sự kiện bằng thuốc phép, hệ số chuỗi ×1→×20 (28/10/2026)</t>
+          <t>Đào báu (Dig &amp; Pharaoh) — Đào báu — một khuôn, nhiều giao diện (Halloween 15 màn, Pharaoh 10 màn) (28/10/2026)</t>
         </is>
       </c>
     </row>
@@ -2949,7 +5147,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Popup Lễ hội Halloween 4d 22h, Tham gia.</t>
+          <t>Popup chủ đề (Halloween / Pharaoh) với đồng hồ và nút Tham gia; tự mở trong chuỗi popup đầu phiên.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -2959,7 +5157,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>HalloweenFestival/01_join_popup</t>
+          <t>DiggingEvents/01_join_popup, DiggingEvents/10_pharaoh_join</t>
         </is>
       </c>
     </row>
@@ -2969,7 +5167,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Xem trước khu hoàn chỉnh</t>
+          <t>Luật 4 bước</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -2979,7 +5177,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Cảnh khu lễ hội đã trang trí đủ, ghi chú “Xem trước trang trí”.</t>
+          <t>Thắng màn → thu cuốc/xẻng → tìm đồ ẩn → giành phần thưởng.</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -2989,7 +5187,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>HalloweenFestival/02_preview_finished_area</t>
+          <t>DiggingEvents/08_info, DiggingEvents/11_pharaoh_how_to</t>
         </is>
       </c>
     </row>
@@ -2999,17 +5197,17 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Luật</t>
+          <t>Bàn đào</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Giao diện</t>
+          <t>Người chơi</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Thu thuốc từ các màn → xây khu → nhận bí ngô → nhận thưởng; dải hệ số ×1…×20, thua về ×1.</t>
+          <t>Màn 1/15 (Halloween) hoặc 1/10 (Pharaoh): khung trên là hình bóng món cần tìm, lưới đất 3×3, số xẻng ở dưới, thanh quà ở trên.</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -3019,7 +5217,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>HalloweenFestival/03_how_to_play</t>
+          <t>DiggingEvents/04_dig_board, DiggingEvents/12_pharaoh_board</t>
         </is>
       </c>
     </row>
@@ -3029,7 +5227,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Bảng xây</t>
+          <t>Đào</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -3039,7 +5237,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Số thuốc hiện có, hệ số hiện tại, lưới hạng mục có giá thuốc, thanh quà bí ngô phía trên.</t>
+          <t>Mỗi chạm tốn 1 xẻng; ô thứ hai lộ một nửa viên kẹo (món chiếm 2 ô).</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -3049,7 +5247,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>HalloweenFestival/04_build_board, HalloweenFestival/05_area_before_build</t>
+          <t>DiggingEvents/05_dig_one, DiggingEvents/06_dig_two</t>
         </is>
       </c>
     </row>
@@ -3059,7 +5257,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Kỳ đã kết thúc</t>
+          <t>Hết xẻng → shop</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -3069,7 +5267,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Một kỳ cũ cùng loại vẫn còn icon “Đã kết thúc” tới khi người chơi mở xem; xem xong icon biến mất.</t>
+          <t>Bấm “+”: 3 gói xẻng 49k / 129k / 249k.</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -3079,114 +5277,144 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>HalloweenFestival/06_ended_instance</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Hạng mục đầu (quan sát)</t>
+          <t>DiggingEvents/07_buy_shovel</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Hết kỳ</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Giao diện</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>“Đã kết thúc — hãy đào ngay”: vẫn vào đào bằng xẻng còn lại.</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>[Playtest]</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>DiggingEvents/03_ended_dig_now</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>Hạng mục</t>
-        </is>
-      </c>
-      <c r="B11" s="1" t="inlineStr">
-        <is>
-          <t>Thuốc</t>
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Kinh tế đào (quan sát 28/10)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Cổng</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="n">
-        <v>400</v>
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>Mục</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="inlineStr">
+        <is>
+          <t>Giá trị</t>
+        </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Prop</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="n">
-        <v>800</v>
+          <t>Số màn đào</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Halloween 15, Pharaoh 10</t>
+        </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Máy ảnh</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="n">
-        <v>1200</v>
+          <t>Chi phí</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>1 xẻng/cuốc mỗi ô</t>
+        </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Khung</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="n">
-        <v>1600</v>
+          <t>Gói xẻng</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>×10 49.000đ · ×30 129.000đ · ×60 249.000đ</t>
+        </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Căn cứ</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="n">
-        <v>2000</v>
+          <t>Gói Pharaoh “chọn một”</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>24.900đ (800 vàng + 5 cuốc) · 49.000đ (+ rương, 10 cuốc) · 69.000đ (+ 3 thẻ, 30 cuốc) · mua tất cả 99.000đ</t>
+        </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Ghế</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="n">
-        <v>2300</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>[Code]  18 hạng mục (numItems), giá và bí ngô thưởng từ BuildingHalloweenStepBuildSheet (server).</t>
+          <t>Nguồn xẻng/cuốc</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>thắng màn, nhiệm vụ ngày, vòng quay may mắn, gói IAP</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Vận dụng cho game khác</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>Vận dụng cho game khác</t>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Viết lõi sự kiện một lần (DiggingBase) rồi đổi giao diện theo mùa: cùng lúc chạy được 2 kỳ (Halloween + Pharaoh) mà không thêm logic.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Cho người chơi xem trước khu hoàn chỉnh ngay khi tham gia: mục tiêu trực quan rõ hơn mọi thanh tiến độ.</t>
+          <t>Cho phần thưởng nhỏ khi đào trượt và cho dùng xẻng dư sau khi kỳ kết thúc: giảm cảm giác “phí tiền mua xẻng”.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Gắn hệ số chuỗi thắng vào tiền tệ sự kiện (thuốc) để mỗi trận thắng liền mạch đáng giá gấp nhiều lần.</t>
+          <t>Rót vật phẩm sự kiện vào mọi nguồn khác (nhiệm vụ ngày, vòng quay) để người không mua vẫn tiến được.</t>
         </is>
       </c>
     </row>
@@ -3215,7 +5443,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Vòng quay may mắn (Lucky Spin) — Vòng quay may mắn — 8 ô, quay bằng quảng cáo, ô thưởng đổi theo sự kiện (28/10/2026)</t>
+          <t>Early Offer (Ưu đãi sớm) — Ưu đãi sớm — chuỗi 5 chức danh cửa hàng, giá gạch, đếm ngược (28/10/2026)</t>
         </is>
       </c>
     </row>
@@ -3257,7 +5485,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Vòng quay</t>
+          <t>Popup offer</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -3267,7 +5495,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Mở từ icon và tự mở sau trận.</t>
+          <t>Store Supervisor Offer.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -3277,7 +5505,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>LuckySpin/01_wheel_ad_spin, LuckySpin/02_auto_open_on_return</t>
+          <t>EarlyOffer/01_store_supervisor_offer</t>
         </is>
       </c>
     </row>
@@ -3291,7 +5519,7 @@
     <row r="7">
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Vòng quay thưởng quảng cáo là nguồn rewarded ổn định; đổi ô thưởng sang vật phẩm sự kiện để nó phục vụ sự kiện đang chạy.</t>
+          <t>Đặt tên gói theo “cấp bậc nghề nghiệp” trong thế giới game: người chơi thấy mình đang thăng tiến chứ không phải đang bị bán hàng.</t>
         </is>
       </c>
     </row>

</xml_diff>